<commit_message>
Add dietary reference intake (DRI 2020) lines to 16-item chart
- New "食事摂取基準" sheet in legends.xlsx with all DRI values
- Green lines: male 18-29y reference; dashed lighter green: male 30-49y
  (only shown when value differs from 18-29y, e.g. calcium 800→750mg)
- Purple lines: female 18-29y reference
- PFC panel: target range bands (P:13-20%E, F:20-30%E, C:50-65%E)
- All values editable via legends.xlsx

https://claude.ai/code/session_01AVgnxSoyf9YpGa1dQKwayT
</commit_message>
<xml_diff>
--- a/legends.xlsx
+++ b/legends.xlsx
@@ -12,6 +12,7 @@
     <sheet name="図2_栄養素" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="食品群ラベル" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="栄養素ラベル" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="食事摂取基準" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +39,11 @@
       <i val="1"/>
       <color rgb="007F7F7F"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -84,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -96,6 +102,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2387,4 +2394,653 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>食事摂取基準 2020年版（推奨量／目安量／目標量）　※空欄＝基準値なし・値を変更する場合はこのシートを編集してください</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>栄養素キー</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>単位</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>種別</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>男性 18-29歳</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>男性 30-49歳</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>女性 18-29歳</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>女性 30-49歳</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>凡例ラベル（男性）</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>凡例ラベル（女性）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>エネルギー</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>kcal/日</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>推定必要量</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2650</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>2700</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>2050</v>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>推定必要量(男)</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>推定必要量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>エネルギー_kg</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>kcal/kg</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>参考値</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>たんぱく質</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>g/日</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>推奨量</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>推奨量(男)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>推奨量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>たんぱく質/kg BW</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>g/kg</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>参考値</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>参考値(男)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>参考値(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>炭水化物</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>g/日</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>目標量(%E換算)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>炭水化物_kg</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>g/kg</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>目標量(%E換算)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>%E</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>目標量（下限）</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>食物繊維総量</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>g/日</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>目安量</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>目安量(男)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>目安量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>食塩相当量</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>g/日</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>目標量(未満)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>目標量(男)</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>目標量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>カルシウム</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>mg/日</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>推奨量</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>750</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>650</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>650</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>推奨量(男)</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>推奨量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>鉄</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>mg/日</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>推奨量</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>推奨量(男)</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>推奨量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ビタミンD</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>µg/日</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>目安量</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>目安量(男)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>目安量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ビタミンB1</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>mg/日</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>推奨量</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>推奨量(男)</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>推奨量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ビタミンB2</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>mg/日</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>推奨量</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>推奨量(男)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>推奨量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>ビタミンB6</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>mg/日</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>推奨量</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>推奨量(男)</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>推奨量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ビタミンC</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>mg/日</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>推奨量</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>推奨量(男)</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>推奨量(女)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>※ エネルギー推定必要量はPAL II（ふつう）の値。たんぱく質/kg BW の参考値は EAR 算定基礎値（0.9g/kg）。炭水化物は目標量が 50〜65%E のため g/日換算なし。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update DRI reference lines to 2025 edition, 18-29y only
- Switch to 食事摂取基準2025年版 (vitamin D updated: 8.5→12.0µg)
- Show only 18-29y lines; remove 30-49y comparison lines
- Remove reference lines for たんぱく質 and 食塩相当量 per request
- Simplify legends.xlsx 食事摂取基準 sheet (drop 30-49y columns)

https://claude.ai/code/session_01AVgnxSoyf9YpGa1dQKwayT
</commit_message>
<xml_diff>
--- a/legends.xlsx
+++ b/legends.xlsx
@@ -2402,24 +2402,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>食事摂取基準 2020年版（推奨量／目安量／目標量）　※空欄＝基準値なし・値を変更する場合はこのシートを編集してください</t>
+          <t>食事摂取基準 2025年版（18〜29歳）　推奨量／目安量／目標量　※空欄＝参照線なし・値を変更する場合はこのシートを編集してください</t>
         </is>
       </c>
     </row>
@@ -2446,25 +2444,15 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>男性 30-49歳</t>
+          <t>女性 18-29歳</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>女性 18-29歳</t>
+          <t>凡例ラベル（男性）</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t>女性 30-49歳</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>凡例ラベル（男性）</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>凡例ラベル（女性）</t>
         </is>
@@ -2490,20 +2478,14 @@
         <v>2650</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>2700</v>
-      </c>
-      <c r="F3" s="3" t="n">
         <v>2000</v>
       </c>
-      <c r="G3" s="3" t="n">
-        <v>2050</v>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>推定必要量(男)</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>推定必要量(女)</t>
         </is>
@@ -2527,10 +2509,8 @@
       </c>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2545,31 +2525,13 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>推奨量</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>65</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>65</v>
-      </c>
-      <c r="F5" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>推奨量(男)</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>推奨量(女)</t>
-        </is>
-      </c>
+          <t>推奨量（参照線なし）</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2587,28 +2549,10 @@
           <t>参考値</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E6" s="2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>参考値(男)</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>参考値(女)</t>
-        </is>
-      </c>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -2628,10 +2572,8 @@
       </c>
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2651,10 +2593,8 @@
       </c>
       <c r="D8" s="2" t="n"/>
       <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2669,15 +2609,13 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>目標量（下限）</t>
+          <t>目標量（帯表示）</t>
         </is>
       </c>
       <c r="D9" s="3" t="n"/>
       <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2699,20 +2637,14 @@
         <v>21</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="F10" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>目安量(男)</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>目安量(女)</t>
         </is>
@@ -2731,31 +2663,13 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>目標量(未満)</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>目標量(男)</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>目標量(女)</t>
-        </is>
-      </c>
+          <t>目標量（参照線なし）</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n"/>
+      <c r="E11" s="3" t="n"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2777,20 +2691,14 @@
         <v>800</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>750</v>
-      </c>
-      <c r="F12" s="2" t="n">
         <v>650</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>650</v>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>推奨量(男)</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>推奨量(女)</t>
         </is>
@@ -2816,20 +2724,14 @@
         <v>7.5</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F13" s="3" t="n">
         <v>10.5</v>
       </c>
-      <c r="G13" s="3" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>推奨量(男)</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>推奨量(女)</t>
         </is>
@@ -2852,23 +2754,17 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>8.5</v>
+        <v>12</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
+        <v>12</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>目安量(男)</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>目安量(女)</t>
         </is>
@@ -2894,20 +2790,14 @@
         <v>1.4</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F15" s="3" t="n">
         <v>1.1</v>
       </c>
-      <c r="G15" s="3" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>推奨量(男)</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>推奨量(女)</t>
         </is>
@@ -2933,20 +2823,14 @@
         <v>1.6</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="F16" s="2" t="n">
         <v>1.2</v>
       </c>
-      <c r="G16" s="2" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>推奨量(男)</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>推奨量(女)</t>
         </is>
@@ -2972,20 +2856,14 @@
         <v>1.4</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F17" s="3" t="n">
         <v>1.1</v>
       </c>
-      <c r="G17" s="3" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>推奨量(男)</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>推奨量(女)</t>
         </is>
@@ -3013,18 +2891,12 @@
       <c r="E18" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="F18" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>推奨量(男)</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>推奨量(女)</t>
         </is>
@@ -3033,13 +2905,13 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>※ エネルギー推定必要量はPAL II（ふつう）の値。たんぱく質/kg BW の参考値は EAR 算定基礎値（0.9g/kg）。炭水化物は目標量が 50〜65%E のため g/日換算なし。</t>
+          <t>※ エネルギーはPAL II（ふつう）。ビタミンD 12.0µg は2025年版改定値（2020年版は8.5µg）。たんぱく質・食塩相当量は参照線を表示しない設定（値をNoneから変更すれば表示されます）。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>